<commit_message>
BLAST Premier 2026 Seoul Stage 2
</commit_message>
<xml_diff>
--- a/file/history.xlsx
+++ b/file/history.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/faa3f9bfbb5dc780/Documentos/GitHub/ck-tools/file/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joao.abraga\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="563" documentId="13_ncr:1_{AB7ADBC0-0AFC-4EB5-BDC6-F57936754D64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{875A5B4F-0713-4E80-888F-0BBE7E743135}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77347E75-C064-47B0-B07A-BDBB4F745A11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2520" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{39BF18F1-6CA4-42F4-B020-2D59954264FB}"/>
+    <workbookView xWindow="4890" yWindow="3630" windowWidth="21600" windowHeight="11295" xr2:uid="{39BF18F1-6CA4-42F4-B020-2D59954264FB}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2786" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2876" uniqueCount="268">
   <si>
     <t>Team 1</t>
   </si>
@@ -966,7 +966,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -12498,148 +12498,364 @@
       </c>
     </row>
     <row r="558" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A558" s="11"/>
-      <c r="B558" s="11"/>
-      <c r="C558" s="11"/>
-      <c r="D558" s="11"/>
-      <c r="E558" s="11"/>
-      <c r="F558" s="11"/>
+      <c r="A558" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="B558" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C558" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D558" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="E558" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F558" s="8">
+        <v>46246</v>
+      </c>
     </row>
     <row r="559" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A559" s="11"/>
-      <c r="B559" s="11"/>
-      <c r="C559" s="11"/>
-      <c r="D559" s="11"/>
-      <c r="E559" s="11"/>
-      <c r="F559" s="11"/>
+      <c r="A559" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="B559" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C559" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D559" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E559" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F559" s="8">
+        <v>46246</v>
+      </c>
     </row>
     <row r="560" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A560" s="11"/>
-      <c r="B560" s="11"/>
-      <c r="C560" s="11"/>
-      <c r="D560" s="11"/>
-      <c r="E560" s="11"/>
-      <c r="F560" s="11"/>
+      <c r="A560" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B560" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C560" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D560" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E560" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F560" s="9">
+        <v>46246</v>
+      </c>
     </row>
     <row r="561" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A561" s="11"/>
-      <c r="B561" s="11"/>
-      <c r="C561" s="11"/>
-      <c r="D561" s="11"/>
-      <c r="E561" s="11"/>
-      <c r="F561" s="11"/>
+      <c r="A561" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B561" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C561" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D561" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E561" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F561" s="9">
+        <v>46246</v>
+      </c>
     </row>
     <row r="562" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A562" s="11"/>
-      <c r="B562" s="11"/>
-      <c r="C562" s="11"/>
-      <c r="D562" s="11"/>
-      <c r="E562" s="11"/>
-      <c r="F562" s="11"/>
+      <c r="A562" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B562" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C562" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="D562" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="E562" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F562" s="9">
+        <v>46246</v>
+      </c>
     </row>
     <row r="563" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A563" s="11"/>
-      <c r="B563" s="11"/>
-      <c r="C563" s="11"/>
-      <c r="D563" s="11"/>
-      <c r="E563" s="11"/>
-      <c r="F563" s="11"/>
+      <c r="A563" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B563" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C563" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D563" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="E563" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F563" s="8">
+        <v>46246</v>
+      </c>
     </row>
     <row r="564" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A564" s="11"/>
-      <c r="B564" s="11"/>
-      <c r="C564" s="11"/>
-      <c r="D564" s="11"/>
-      <c r="E564" s="11"/>
-      <c r="F564" s="11"/>
+      <c r="A564" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B564" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C564" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D564" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E564" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F564" s="8">
+        <v>46246</v>
+      </c>
     </row>
     <row r="565" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A565" s="11"/>
-      <c r="B565" s="11"/>
-      <c r="C565" s="11"/>
-      <c r="D565" s="11"/>
-      <c r="E565" s="11"/>
-      <c r="F565" s="11"/>
+      <c r="A565" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B565" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C565" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D565" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E565" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F565" s="8">
+        <v>46246</v>
+      </c>
     </row>
     <row r="566" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A566" s="11"/>
-      <c r="B566" s="11"/>
-      <c r="C566" s="11"/>
-      <c r="D566" s="11"/>
-      <c r="E566" s="11"/>
-      <c r="F566" s="11"/>
+      <c r="A566" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B566" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C566" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D566" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="E566" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F566" s="9">
+        <v>46246</v>
+      </c>
     </row>
     <row r="567" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A567" s="11"/>
-      <c r="B567" s="11"/>
-      <c r="C567" s="11"/>
-      <c r="D567" s="11"/>
-      <c r="E567" s="11"/>
-      <c r="F567" s="11"/>
+      <c r="A567" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B567" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C567" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D567" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="E567" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F567" s="9">
+        <v>46246</v>
+      </c>
     </row>
     <row r="568" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A568" s="11"/>
-      <c r="B568" s="11"/>
-      <c r="C568" s="11"/>
-      <c r="D568" s="11"/>
-      <c r="E568" s="11"/>
-      <c r="F568" s="11"/>
+      <c r="A568" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B568" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C568" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D568" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E568" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F568" s="8">
+        <v>46247</v>
+      </c>
     </row>
     <row r="569" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A569" s="11"/>
-      <c r="B569" s="11"/>
-      <c r="C569" s="11"/>
-      <c r="D569" s="11"/>
-      <c r="E569" s="11"/>
-      <c r="F569" s="11"/>
+      <c r="A569" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B569" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C569" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D569" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="E569" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F569" s="8">
+        <v>46247</v>
+      </c>
     </row>
     <row r="570" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A570" s="11"/>
-      <c r="B570" s="11"/>
-      <c r="C570" s="11"/>
-      <c r="D570" s="11"/>
-      <c r="E570" s="11"/>
-      <c r="F570" s="11"/>
+      <c r="A570" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B570" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C570" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D570" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E570" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F570" s="9">
+        <v>46247</v>
+      </c>
     </row>
     <row r="571" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A571" s="11"/>
-      <c r="B571" s="11"/>
-      <c r="C571" s="11"/>
-      <c r="D571" s="11"/>
-      <c r="E571" s="11"/>
-      <c r="F571" s="11"/>
+      <c r="A571" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B571" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C571" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D571" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E571" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F571" s="9">
+        <v>46247</v>
+      </c>
     </row>
     <row r="572" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A572" s="11"/>
-      <c r="B572" s="11"/>
-      <c r="C572" s="11"/>
-      <c r="D572" s="11"/>
-      <c r="E572" s="11"/>
-      <c r="F572" s="11"/>
+      <c r="A572" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="B572" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C572" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D572" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="E572" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F572" s="8">
+        <v>46247</v>
+      </c>
     </row>
     <row r="573" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A573" s="11"/>
-      <c r="B573" s="11"/>
-      <c r="C573" s="11"/>
-      <c r="D573" s="11"/>
-      <c r="E573" s="11"/>
-      <c r="F573" s="11"/>
+      <c r="A573" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="B573" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C573" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D573" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E573" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F573" s="8">
+        <v>46247</v>
+      </c>
     </row>
     <row r="574" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A574" s="11"/>
-      <c r="B574" s="11"/>
-      <c r="C574" s="11"/>
-      <c r="D574" s="11"/>
-      <c r="E574" s="11"/>
-      <c r="F574" s="11"/>
+      <c r="A574" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B574" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C574" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D574" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E574" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F574" s="9">
+        <v>46247</v>
+      </c>
     </row>
     <row r="575" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A575" s="11"/>
-      <c r="B575" s="11"/>
-      <c r="C575" s="11"/>
-      <c r="D575" s="11"/>
-      <c r="E575" s="11"/>
-      <c r="F575" s="11"/>
+      <c r="A575" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B575" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C575" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D575" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E575" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F575" s="9">
+        <v>46247</v>
+      </c>
     </row>
     <row r="576" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A576" s="11"/>

</xml_diff>